<commit_message>
Update models to only use User table instead of Doctor and Patient
</commit_message>
<xml_diff>
--- a/Schema/romandi_vadaszhaz_klinika_mongodb_struktura.xlsx
+++ b/Schema/romandi_vadaszhaz_klinika_mongodb_struktura.xlsx
@@ -5,27 +5,25 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programozás\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programozás\Klinik\romandi-vadaszhaz-klinik-backend\Schema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6824C524-E9A7-46E6-B53A-44ECDD1B3000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE58A95C-EC5D-4E11-B0AB-DD3E07C79EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="users" sheetId="1" r:id="rId1"/>
-    <sheet name="doctors" sheetId="2" r:id="rId2"/>
-    <sheet name="patients" sheetId="3" r:id="rId3"/>
-    <sheet name="appointments" sheetId="4" r:id="rId4"/>
-    <sheet name="services" sheetId="6" r:id="rId5"/>
-    <sheet name="records" sheetId="5" r:id="rId6"/>
+    <sheet name="appointments" sheetId="4" r:id="rId2"/>
+    <sheet name="services" sheetId="6" r:id="rId3"/>
+    <sheet name="records" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="56">
   <si>
     <t>Mező</t>
   </si>
@@ -93,46 +91,7 @@
     <t>user_id</t>
   </si>
   <si>
-    <t>Kapcsolt user</t>
-  </si>
-  <si>
     <t>users._id</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>Orvos neve</t>
-  </si>
-  <si>
-    <t>specialization</t>
-  </si>
-  <si>
-    <t>Szakterület</t>
-  </si>
-  <si>
-    <t>phone</t>
-  </si>
-  <si>
-    <t>Telefonszám</t>
-  </si>
-  <si>
-    <t>Aktív orvos</t>
-  </si>
-  <si>
-    <t>Páciens neve</t>
-  </si>
-  <si>
-    <t>birthDate</t>
-  </si>
-  <si>
-    <t>Születési dátum</t>
-  </si>
-  <si>
-    <t>address</t>
-  </si>
-  <si>
-    <t>Lakcím</t>
   </si>
   <si>
     <t>doctor_id</t>
@@ -666,198 +625,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" t="s">
-        <v>35</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -889,30 +656,30 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D4" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -923,32 +690,32 @@
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
         <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -967,7 +734,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8192EC-9D82-48D5-95BA-C6BC6902A63D}">
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1005,99 +772,99 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="C7" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="D9" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1105,10 +872,10 @@
         <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1116,7 +883,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1151,55 +918,55 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="D5" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1210,7 +977,7 @@
         <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>